<commit_message>
Templates: Templates thread's regenerated manifest (Hook Bank's 60 hooks, Eli-reviewed flags) and files
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EiAPcndz9mZ73fvAWuA5p3
</commit_message>
<xml_diff>
--- a/content/templates/files/hook-bank/127-hook-bank-example.xlsx
+++ b/content/templates/files/hook-bank/127-hook-bank-example.xlsx
@@ -16,13 +16,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Winners" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hook bank'!$A$3:$D$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hook bank'!$A$3:$F$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Hook bank'!$3:$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'My hooks'!$A$3:$J$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'My hooks'!$3:$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Captions'!$A$3:$C$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Captions'!$3:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CTAs'!$A$3:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'CTAs'!$A$3:$C$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'CTAs'!$3:$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Winners'!$A$3:$G$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Winners'!$3:$3</definedName>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B29"/>
+  <dimension ref="B2:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -670,7 +670,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>42 fill-in-the-blank hooks, 10 caption templates and 10 calls to action, plus a log that shows which hook type works for your audience.</t>
+          <t>60 fill-in-the-blank hooks with a filled example each, 10 caption templates and 10 calls to action, plus a log that shows which hook type works for you.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
     <row r="9" ht="32" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>1.  Browse the Hook bank tab. Filter by type: story, mistake, contrarian, how-to, result, behind the scenes.</t>
+          <t>1.  Browse the Hook bank tab. Filter by type: story, mistake, contrarian, how-to, list, result, behind the scenes, call-out, comparison, experiment. Each hook has a filled example.</t>
         </is>
       </c>
     </row>
@@ -793,15 +793,22 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="11" t="inlineStr">
+    <row r="28" ht="30" customHeight="1">
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Contrarian, result and experiment hooks only when they're true: you believe it, the result is real, you ran the test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Make today day one.  ·  127group.io</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="12" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Template drafted from Eli Christiansen's frameworks. © 127 Group LLC. For your own business use.</t>
         </is>
@@ -818,13 +825,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -859,7 +868,17 @@
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
+          <t>Filled example</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
           <t>Works for pillar</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Rule</t>
         </is>
       </c>
     </row>
@@ -874,14 +893,20 @@
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>I started [business] with [small amount or resource]. Here's what happened.</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
+          <t>I started [business] with [small amount or resource]. Here's what month one looked like.</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>I started a sneaker cleaning business with $60 and a toothbrush.</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F4" s="17" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="16" t="n">
@@ -894,14 +919,20 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>A year ago I was [old situation]. Today I'm [new situation].</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
+          <t>[Time] ago I [old situation]. Now I [new situation].</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Six months ago I couldn't edit a video. Now I edit for 4 podcasts.</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F5" s="17" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="16" t="n">
@@ -914,14 +945,20 @@
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>The day I almost quit [thing] was the day [turning point].</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
+          <t>The day I almost quit [thing], [what happened].</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>The day I almost quit making candles, a local shop asked to stock them.</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F6" s="17" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
@@ -934,14 +971,20 @@
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>My first customer for [offer] came from [unexpected place].</t>
-        </is>
-      </c>
-      <c r="D7" s="16" t="inlineStr">
+          <t>My first customer came from [unexpected place].</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>My first resume client came from a comment I left on a Reddit thread.</t>
+        </is>
+      </c>
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F7" s="17" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="16" t="n">
@@ -954,14 +997,20 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>Nobody believed [thing] would work. Here's what I did anyway.</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
+          <t>Everyone told me [doubt]. Here's what happened when I tried anyway.</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Everyone told me college students won't pay for meal prep.</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F8" s="17" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
@@ -974,14 +1023,20 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>This is what [number] weeks of building [business] looks like.</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
+          <t>This is what [number] weeks of building [business] actually looks like.</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>This is what 8 weeks of building a phone repair business actually looks like.</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>You</t>
         </is>
       </c>
+      <c r="F9" s="17" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="16" t="n">
@@ -989,19 +1044,25 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Mistake</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>I didn't think I was qualified to [goal]. Here's what changed.</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>You</t>
-        </is>
-      </c>
+          <t>I wasted [time or money] on [thing] so you don't have to.</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>I wasted $200 on cleaning kits so you don't have to.</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>Teach or You</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
@@ -1014,14 +1075,20 @@
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>I wasted [time or money] on [thing] so you don't have to.</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
+          <t>Stop [common action] if you want [result].</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>Stop washing suede with water if you want it to last.</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Teach or You</t>
         </is>
       </c>
+      <c r="F11" s="17" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="16" t="n">
@@ -1034,14 +1101,20 @@
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>The biggest mistake I made starting [business]: [mistake].</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
+          <t>[Number] mistakes I made in my first [timeframe] of [business].</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>3 mistakes I made in my first month of selling candles.</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Teach or You</t>
         </is>
       </c>
+      <c r="F12" s="17" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
@@ -1054,14 +1127,20 @@
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Stop [common action] if you want [result].</t>
-        </is>
-      </c>
-      <c r="D13" s="16" t="inlineStr">
+          <t>If you're still [common habit], you're losing [result].</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>If you're still pricing by the hour, you're losing your best clients.</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Teach or You</t>
         </is>
       </c>
+      <c r="F13" s="17" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="16" t="n">
@@ -1074,14 +1153,20 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>[Number] mistakes I made in my first [timeframe] of [business].</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
+          <t>Don't [action] until you've [done this first].</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>Don't print 500 stickers until you've sold 50.</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Teach or You</t>
         </is>
       </c>
+      <c r="F14" s="17" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
@@ -1094,14 +1179,20 @@
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>If you're doing [common habit], you're losing [result].</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
+          <t>The [mistake] almost every [person] makes with [thing].</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>The mistake almost every new seller makes with shipping costs.</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>Teach or You</t>
         </is>
       </c>
+      <c r="F15" s="17" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n">
@@ -1109,17 +1200,27 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>Mistake</t>
+          <t>Contrarian</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>I tried [popular advice]. It didn't work. Here's why.</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="inlineStr">
-        <is>
-          <t>Teach or You</t>
+          <t>Unpopular opinion: you don't need [common belief] to [result].</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Unpopular opinion: you don't need a camera to start a video editing business.</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1230,27 @@
       </c>
       <c r="B17" s="16" t="inlineStr">
         <is>
-          <t>Mistake</t>
+          <t>Contrarian</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>Don't [action] until you've done this first.</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="inlineStr">
-        <is>
-          <t>Teach or You</t>
+          <t>Everyone says [advice]. Here's why I stopped.</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>Everyone says post every day. Here's why I post 3 times a week.</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1265,22 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>Unpopular opinion: you don't need [common belief] to [result].</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="inlineStr">
+          <t>[Popular thing] is overrated for [person]. Do this instead.</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>Meal kits are overrated for college students.</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1295,22 @@
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>Everyone says [advice]. I think that's wrong.</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="inlineStr">
+          <t>You don't have a [surface problem] problem. You have a [real problem] problem.</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>You don't have a views problem. You have a first-2-seconds problem.</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1194,12 +1325,22 @@
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>[Popular thing] is overrated. Do this instead.</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
+          <t>[Thing people fear] isn't the hard part. [Real hard part] is.</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Getting your first client isn't the hard part. Getting your second one is.</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1355,22 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>The worst advice I got about [topic]: [advice].</t>
-        </is>
-      </c>
-      <c r="D21" s="16" t="inlineStr">
+          <t>The worst advice I got about [topic] was [advice].</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>The worst advice I got about pricing was to start cheap and raise it later.</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
+        </is>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
+        <is>
+          <t>Only if you believe it and back it up in the post</t>
         </is>
       </c>
     </row>
@@ -1229,19 +1380,25 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>Contrarian</t>
+          <t>How-to</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>You don't have a [problem] problem. You have a [real problem] problem.</t>
-        </is>
-      </c>
-      <c r="D22" s="16" t="inlineStr">
+          <t>How to [result] in [timeframe] without [pain].</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>How to clean white midsoles in 5 minutes without bleach.</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F22" s="17" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n">
@@ -1249,19 +1406,25 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>Contrarian</t>
+          <t>How-to</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>Nobody talks about this part of [topic].</t>
-        </is>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
+          <t>Here's exactly how I'd [result] if I started today.</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>Here's exactly how I'd get my first editing client if I started today.</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F23" s="17" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="16" t="n">
@@ -1269,19 +1432,25 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>Contrarian</t>
+          <t>How-to</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>[Thing people fear] isn't the hard part. [Real hard part] is.</t>
-        </is>
-      </c>
-      <c r="D24" s="16" t="inlineStr">
+          <t>The [number]-minute fix for [problem].</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>The 2-minute fix for a resume that gets no replies.</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F24" s="17" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="16" t="n">
@@ -1294,14 +1463,20 @@
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>How to [result] in [timeframe] without [pain].</t>
-        </is>
-      </c>
-      <c r="D25" s="16" t="inlineStr">
+          <t>How I [result] using only [tool or phone].</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>How I film product videos using only my phone and a window.</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F25" s="17" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="16" t="n">
@@ -1314,14 +1489,20 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>Here's exactly how I'd [result] if I started today.</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr">
+          <t>Do this before you [common action].</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Do this before you send your first invoice.</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F26" s="17" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n">
@@ -1334,14 +1515,20 @@
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>[Number] steps to [result]. Save this.</t>
-        </is>
-      </c>
-      <c r="D27" s="16" t="inlineStr">
+          <t>The easiest way to [result] if you're [specific situation].</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>The easiest way to meal prep if you live in a dorm with no stove.</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F27" s="17" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="16" t="n">
@@ -1349,19 +1536,25 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>How-to</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>The [number]-minute fix for [problem].</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
+          <t>[Number] [things] I tested, ranked from worst to best.</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>5 sneaker cleaners I tested, ranked from worst to best.</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F28" s="17" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="16" t="n">
@@ -1369,19 +1562,25 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>How-to</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>How I [result] using only [tool or phone].</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
+          <t>[Number] free tools I use every week to [result].</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>4 free tools I use every week to run my tutoring business.</t>
+        </is>
+      </c>
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F29" s="17" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="16" t="n">
@@ -1389,19 +1588,25 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>How-to</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>Do this before you [common action].</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
+          <t>[Number] signs your [thing] is [problem].</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>3 signs your resume is getting filtered out before a human sees it.</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F30" s="17" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="n">
@@ -1409,19 +1614,25 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>How-to</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>The easiest way to [result] for [specific person].</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr">
+          <t>[Number] things I wish I knew before [milestone].</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>3 things I wish I knew before my first market stall.</t>
+        </is>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Teach</t>
         </is>
       </c>
+      <c r="F31" s="17" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="n">
@@ -1429,19 +1640,25 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>This [before] became [after] in [timeframe].</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Proof</t>
-        </is>
-      </c>
+          <t>[Number] [things] under [$ amount] that [result].</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>3 lighting setups under $20 that make phone videos look professional.</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="n">
@@ -1449,19 +1666,25 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>List</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>How [customer type] went from [before] to [after].</t>
-        </is>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
-        <is>
-          <t>Proof</t>
-        </is>
-      </c>
+          <t>My [number]-step [process] for [result]. Copy it.</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>My 4-step packing checklist for orders that never arrive broken.</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="16" t="n">
@@ -1474,12 +1697,22 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>What [price or amount] gets you with [offer].</t>
-        </is>
-      </c>
-      <c r="D34" s="16" t="inlineStr">
+          <t>This [before] became [after] in [timeframe].</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>This yellowed midsole went white again in 20 minutes.</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Proof</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1494,12 +1727,22 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>We just [milestone]. Here's what actually made the difference.</t>
-        </is>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
+          <t>How [customer type] went from [before] to [after].</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>How a nursing student went from 0 interview calls to 3 in two weeks.</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Proof</t>
+        </is>
+      </c>
+      <c r="F35" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1757,22 @@
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>Watch this [thing] go from [before] to [after].</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
+          <t>What [price] gets you with [offer].</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>What $25 gets you with my resume review.</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Proof</t>
+        </is>
+      </c>
+      <c r="F36" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1534,12 +1787,22 @@
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>[Customer] said [exact quote]. Here's what we did.</t>
-        </is>
-      </c>
-      <c r="D37" s="16" t="inlineStr">
+          <t>[Customer] said "[exact words]." Here's what we did.</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>A client said "I finally get algebra." Here's what we changed.</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Proof</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1554,12 +1817,22 @@
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>My [first / tenth / best] [sale, client, drop] and what I learned.</t>
-        </is>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
+          <t>My [first, 10th or 100th] [sale, client or order] and what it taught me.</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>My 10th order and the packing mistake it exposed.</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>Proof</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1569,17 +1842,27 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>Behind the scenes</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>A day running [business] while [other commitment].</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>You or Proof</t>
+          <t>Watch this [thing] go from [before] to [after].</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Watch this $8 thrifted jacket go from stained to resale ready.</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>Real results only: yours, or a customer's shared with permission</t>
         </is>
       </c>
     </row>
@@ -1594,14 +1877,20 @@
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>What goes into one [product or service] that nobody sees.</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
+          <t>A day running [business] while [other commitment].</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>A day running a candle business while working a full-time job.</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F40" s="17" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="16" t="n">
@@ -1614,14 +1903,20 @@
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>Packing orders for [business]. Come with me.</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
+          <t>What goes into one [product or service] that nobody sees.</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>What goes into one $30 logo that nobody sees.</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F41" s="17" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="n">
@@ -1634,14 +1929,20 @@
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>Here's what my [setup / workspace / process] actually looks like.</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
+          <t>Packing [number] orders for [business]. Come with me.</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>Packing 14 orders for my sticker shop.</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F42" s="17" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="n">
@@ -1654,14 +1955,20 @@
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>The part of [business] I hate, and why I do it anyway.</t>
-        </is>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
+          <t>Here's what my [setup or process] actually looks like.</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>Here's what my $0 editing setup actually looks like.</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="16" t="n">
@@ -1677,11 +1984,17 @@
           <t>Honest update: week [number] of building [business].</t>
         </is>
       </c>
-      <c r="D44" s="16" t="inlineStr">
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>Honest update: week 6 of building a meal prep business.</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F44" s="17" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="n">
@@ -1694,20 +2007,518 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>Here's how a [service] session actually goes.</t>
-        </is>
-      </c>
-      <c r="D45" s="16" t="inlineStr">
+          <t>The part of [business] I hate, and why I do it anyway.</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>The part of tutoring I hate, and why I do it anyway.</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="inlineStr">
         <is>
           <t>You or Proof</t>
         </is>
       </c>
+      <c r="F45" s="17" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="n">
+        <v>43</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>If you're a [specific person] who [situation], this is for you.</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>If you're a student athlete who hates cooking, this is for you.</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F46" s="17" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>This is for every [person] who's tired of [pain].</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>This is for every freelancer who's tired of chasing invoices.</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>Do you [common behavior]? Here's what it's doing to [thing].</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Do you machine-wash your sneakers? Here's what it's doing to the glue.</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="n">
+        <v>46</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>Raise your hand if you've ever [relatable pain].</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Raise your hand if you've ever bought a planner and quit by February.</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="n">
+        <v>47</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>Only watch this if you [qualifier].</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Only watch this if you sell something under $50.</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n">
+        <v>48</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>POV: you [relatable moment].</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>POV: you finally clean the sneakers you've been hiding in your closet.</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Teach</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n">
+        <v>49</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>[Option A] vs [option B]: which one actually [result]?</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>$5 cleaner vs $25 cleaner: which one actually works?</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>I tested [cheap thing] and [expensive thing] for [timeframe]. Here's the verdict.</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>I tested a $12 and a $60 ring light for a week.</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>What [amount] gets you at [place A] vs [place B].</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>What $50 gets you at a local print shop vs online.</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="n">
+        <v>52</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>Beginner [thing] vs pro [thing], same [tool].</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Beginner lighting vs pro lighting, same phone.</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>53</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>[Task] the slow way vs the fast way.</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Packing orders the slow way vs the fast way.</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>What [customers] expect vs what actually happens.</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>What clients expect from a logo designer vs what actually happens.</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>Teach or Proof</t>
+        </is>
+      </c>
+      <c r="F57" s="17" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="16" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>I tried [thing] for [timeframe]. Here's what happened.</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>I sold at a farmers market for 4 weekends.</t>
+        </is>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n">
+        <v>56</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>Can you [result] with only [constraint]? Let's find out.</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>Can you start a business with only $50?</t>
+        </is>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>I let [person or group] decide [thing] for my business.</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>I let my followers pick my next candle scent.</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>58</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>Testing [popular claim] so you don't have to.</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>Testing the viral toothpaste sneaker trick so you don't have to.</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F61" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>Day [number] of [challenge].</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>Day 1 of turning $100 into a real business.</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F62" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>I [did something unusual] to get [result]. Was it worth it?</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>I handed out 100 flyers to find tutoring clients.</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>Proof or You</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="inlineStr">
+        <is>
+          <t>Only if you ran it, and show the real outcome</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D45"/>
+  <autoFilter ref="A3:F63"/>
   <dataValidations count="1">
-    <dataValidation sqref="B4:B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Story,Mistake,Contrarian,How-to,Result,Behind the scenes"</formula1>
+    <dataValidation sqref="B4:B63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Story,Mistake,Contrarian,How-to,List,Result,Behind the scenes,Call-out,Comparison,Experiment"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1809,10 +2620,10 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B4,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B4,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D4" s="16" t="inlineStr">
@@ -1850,10 +2661,10 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C5" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B5,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B5,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D5" s="16" t="inlineStr">
@@ -1891,10 +2702,10 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C6" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B6,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B6,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -1932,10 +2743,10 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B7,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B7,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -1973,10 +2784,10 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B8,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B8,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D8" s="16" t="inlineStr">
@@ -2014,10 +2825,10 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B9,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B9,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -2052,7 +2863,7 @@
       <c r="A10" s="17" t="n"/>
       <c r="B10" s="19" t="n"/>
       <c r="C10" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B10,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B10,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D10" s="16" t="n"/>
@@ -2070,7 +2881,7 @@
       <c r="A11" s="17" t="n"/>
       <c r="B11" s="19" t="n"/>
       <c r="C11" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B11,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B11,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D11" s="16" t="n"/>
@@ -2088,7 +2899,7 @@
       <c r="A12" s="17" t="n"/>
       <c r="B12" s="19" t="n"/>
       <c r="C12" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B12,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B12,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D12" s="16" t="n"/>
@@ -2106,7 +2917,7 @@
       <c r="A13" s="17" t="n"/>
       <c r="B13" s="19" t="n"/>
       <c r="C13" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B13,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B13,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D13" s="16" t="n"/>
@@ -2124,7 +2935,7 @@
       <c r="A14" s="17" t="n"/>
       <c r="B14" s="19" t="n"/>
       <c r="C14" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B14,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B14,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D14" s="16" t="n"/>
@@ -2142,7 +2953,7 @@
       <c r="A15" s="17" t="n"/>
       <c r="B15" s="19" t="n"/>
       <c r="C15" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B15,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B15,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D15" s="16" t="n"/>
@@ -2160,7 +2971,7 @@
       <c r="A16" s="17" t="n"/>
       <c r="B16" s="19" t="n"/>
       <c r="C16" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B16,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B16,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D16" s="16" t="n"/>
@@ -2178,7 +2989,7 @@
       <c r="A17" s="17" t="n"/>
       <c r="B17" s="19" t="n"/>
       <c r="C17" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B17,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B17,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D17" s="16" t="n"/>
@@ -2196,7 +3007,7 @@
       <c r="A18" s="17" t="n"/>
       <c r="B18" s="19" t="n"/>
       <c r="C18" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B18,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B18,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D18" s="16" t="n"/>
@@ -2214,7 +3025,7 @@
       <c r="A19" s="17" t="n"/>
       <c r="B19" s="19" t="n"/>
       <c r="C19" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B19,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B19,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D19" s="16" t="n"/>
@@ -2232,7 +3043,7 @@
       <c r="A20" s="17" t="n"/>
       <c r="B20" s="19" t="n"/>
       <c r="C20" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B20,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B20,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D20" s="16" t="n"/>
@@ -2250,7 +3061,7 @@
       <c r="A21" s="17" t="n"/>
       <c r="B21" s="19" t="n"/>
       <c r="C21" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B21,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B21,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D21" s="16" t="n"/>
@@ -2268,7 +3079,7 @@
       <c r="A22" s="17" t="n"/>
       <c r="B22" s="19" t="n"/>
       <c r="C22" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B22,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B22,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D22" s="16" t="n"/>
@@ -2286,7 +3097,7 @@
       <c r="A23" s="17" t="n"/>
       <c r="B23" s="19" t="n"/>
       <c r="C23" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B23,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B23,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D23" s="16" t="n"/>
@@ -2304,7 +3115,7 @@
       <c r="A24" s="17" t="n"/>
       <c r="B24" s="19" t="n"/>
       <c r="C24" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B24,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B24,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D24" s="16" t="n"/>
@@ -2322,7 +3133,7 @@
       <c r="A25" s="17" t="n"/>
       <c r="B25" s="19" t="n"/>
       <c r="C25" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B25,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B25,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D25" s="16" t="n"/>
@@ -2340,7 +3151,7 @@
       <c r="A26" s="17" t="n"/>
       <c r="B26" s="19" t="n"/>
       <c r="C26" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B26,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B26,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D26" s="16" t="n"/>
@@ -2358,7 +3169,7 @@
       <c r="A27" s="17" t="n"/>
       <c r="B27" s="19" t="n"/>
       <c r="C27" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B27,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B27,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D27" s="16" t="n"/>
@@ -2376,7 +3187,7 @@
       <c r="A28" s="17" t="n"/>
       <c r="B28" s="19" t="n"/>
       <c r="C28" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B28,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B28,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D28" s="16" t="n"/>
@@ -2394,7 +3205,7 @@
       <c r="A29" s="17" t="n"/>
       <c r="B29" s="19" t="n"/>
       <c r="C29" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B29,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B29,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D29" s="16" t="n"/>
@@ -2412,7 +3223,7 @@
       <c r="A30" s="17" t="n"/>
       <c r="B30" s="19" t="n"/>
       <c r="C30" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B30,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B30,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D30" s="16" t="n"/>
@@ -2430,7 +3241,7 @@
       <c r="A31" s="17" t="n"/>
       <c r="B31" s="19" t="n"/>
       <c r="C31" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B31,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B31,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D31" s="16" t="n"/>
@@ -2448,7 +3259,7 @@
       <c r="A32" s="17" t="n"/>
       <c r="B32" s="19" t="n"/>
       <c r="C32" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B32,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B32,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D32" s="16" t="n"/>
@@ -2466,7 +3277,7 @@
       <c r="A33" s="17" t="n"/>
       <c r="B33" s="19" t="n"/>
       <c r="C33" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B33,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B33,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D33" s="16" t="n"/>
@@ -2484,7 +3295,7 @@
       <c r="A34" s="17" t="n"/>
       <c r="B34" s="19" t="n"/>
       <c r="C34" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B34,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B34,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D34" s="16" t="n"/>
@@ -2502,7 +3313,7 @@
       <c r="A35" s="17" t="n"/>
       <c r="B35" s="19" t="n"/>
       <c r="C35" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B35,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B35,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D35" s="16" t="n"/>
@@ -2520,7 +3331,7 @@
       <c r="A36" s="17" t="n"/>
       <c r="B36" s="19" t="n"/>
       <c r="C36" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B36,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B36,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D36" s="16" t="n"/>
@@ -2538,7 +3349,7 @@
       <c r="A37" s="17" t="n"/>
       <c r="B37" s="19" t="n"/>
       <c r="C37" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B37,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B37,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D37" s="16" t="n"/>
@@ -2556,7 +3367,7 @@
       <c r="A38" s="17" t="n"/>
       <c r="B38" s="19" t="n"/>
       <c r="C38" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B38,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B38,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D38" s="16" t="n"/>
@@ -2574,7 +3385,7 @@
       <c r="A39" s="17" t="n"/>
       <c r="B39" s="19" t="n"/>
       <c r="C39" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B39,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B39,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D39" s="16" t="n"/>
@@ -2592,7 +3403,7 @@
       <c r="A40" s="17" t="n"/>
       <c r="B40" s="19" t="n"/>
       <c r="C40" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B40,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B40,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D40" s="16" t="n"/>
@@ -2610,7 +3421,7 @@
       <c r="A41" s="17" t="n"/>
       <c r="B41" s="19" t="n"/>
       <c r="C41" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B41,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B41,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D41" s="16" t="n"/>
@@ -2628,7 +3439,7 @@
       <c r="A42" s="17" t="n"/>
       <c r="B42" s="19" t="n"/>
       <c r="C42" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B42,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B42,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D42" s="16" t="n"/>
@@ -2646,7 +3457,7 @@
       <c r="A43" s="17" t="n"/>
       <c r="B43" s="19" t="n"/>
       <c r="C43" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B43,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B43,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D43" s="16" t="n"/>
@@ -2664,7 +3475,7 @@
       <c r="A44" s="17" t="n"/>
       <c r="B44" s="19" t="n"/>
       <c r="C44" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B44,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B44,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D44" s="16" t="n"/>
@@ -2682,7 +3493,7 @@
       <c r="A45" s="17" t="n"/>
       <c r="B45" s="19" t="n"/>
       <c r="C45" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B45,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B45,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D45" s="16" t="n"/>
@@ -2700,7 +3511,7 @@
       <c r="A46" s="17" t="n"/>
       <c r="B46" s="19" t="n"/>
       <c r="C46" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B46,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B46,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D46" s="16" t="n"/>
@@ -2718,7 +3529,7 @@
       <c r="A47" s="17" t="n"/>
       <c r="B47" s="19" t="n"/>
       <c r="C47" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B47,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B47,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D47" s="16" t="n"/>
@@ -2736,7 +3547,7 @@
       <c r="A48" s="17" t="n"/>
       <c r="B48" s="19" t="n"/>
       <c r="C48" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B48,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B48,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D48" s="16" t="n"/>
@@ -2754,7 +3565,7 @@
       <c r="A49" s="17" t="n"/>
       <c r="B49" s="19" t="n"/>
       <c r="C49" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B49,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B49,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D49" s="16" t="n"/>
@@ -2772,7 +3583,7 @@
       <c r="A50" s="17" t="n"/>
       <c r="B50" s="19" t="n"/>
       <c r="C50" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B50,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B50,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D50" s="16" t="n"/>
@@ -2790,7 +3601,7 @@
       <c r="A51" s="17" t="n"/>
       <c r="B51" s="19" t="n"/>
       <c r="C51" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B51,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B51,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D51" s="16" t="n"/>
@@ -2808,7 +3619,7 @@
       <c r="A52" s="17" t="n"/>
       <c r="B52" s="19" t="n"/>
       <c r="C52" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B52,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B52,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D52" s="16" t="n"/>
@@ -2826,7 +3637,7 @@
       <c r="A53" s="17" t="n"/>
       <c r="B53" s="19" t="n"/>
       <c r="C53" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B53,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B53,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D53" s="16" t="n"/>
@@ -2844,7 +3655,7 @@
       <c r="A54" s="17" t="n"/>
       <c r="B54" s="19" t="n"/>
       <c r="C54" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B54,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B54,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D54" s="16" t="n"/>
@@ -2862,7 +3673,7 @@
       <c r="A55" s="17" t="n"/>
       <c r="B55" s="19" t="n"/>
       <c r="C55" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B55,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B55,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D55" s="16" t="n"/>
@@ -2880,7 +3691,7 @@
       <c r="A56" s="17" t="n"/>
       <c r="B56" s="19" t="n"/>
       <c r="C56" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B56,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B56,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D56" s="16" t="n"/>
@@ -2898,7 +3709,7 @@
       <c r="A57" s="17" t="n"/>
       <c r="B57" s="19" t="n"/>
       <c r="C57" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B57,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B57,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D57" s="16" t="n"/>
@@ -2916,7 +3727,7 @@
       <c r="A58" s="17" t="n"/>
       <c r="B58" s="19" t="n"/>
       <c r="C58" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B58,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B58,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D58" s="16" t="n"/>
@@ -2934,7 +3745,7 @@
       <c r="A59" s="17" t="n"/>
       <c r="B59" s="19" t="n"/>
       <c r="C59" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B59,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B59,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D59" s="16" t="n"/>
@@ -2952,7 +3763,7 @@
       <c r="A60" s="17" t="n"/>
       <c r="B60" s="19" t="n"/>
       <c r="C60" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B60,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B60,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D60" s="16" t="n"/>
@@ -2970,7 +3781,7 @@
       <c r="A61" s="17" t="n"/>
       <c r="B61" s="19" t="n"/>
       <c r="C61" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B61,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B61,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D61" s="16" t="n"/>
@@ -2988,7 +3799,7 @@
       <c r="A62" s="17" t="n"/>
       <c r="B62" s="19" t="n"/>
       <c r="C62" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B62,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B62,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D62" s="16" t="n"/>
@@ -3006,7 +3817,7 @@
       <c r="A63" s="17" t="n"/>
       <c r="B63" s="19" t="n"/>
       <c r="C63" s="20">
-        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$45,MATCH(B63,'Hook bank'!$A$4:$A$45,0)),"")</f>
+        <f>IFERROR(INDEX('Hook bank'!$B$4:$B$63,MATCH(B63,'Hook bank'!$A$4:$A$63,0)),"")</f>
         <v/>
       </c>
       <c r="D63" s="16" t="n"/>
@@ -3096,12 +3907,15 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Quick lesson</t>
+          <t>PAS: Problem, agitate, solve</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>[Hook restated]. Here's what I learned: [lesson in one sentence]. [CTA]</t>
+          <t>[The problem, in your customer's words.]
+[Why it's worse than it looks, one specific line.]
+[Your fix, in one or two sentences.]
+[CTA]</t>
         </is>
       </c>
     </row>
@@ -3111,10 +3925,61 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
+          <t>BAB: Before, after, bridge</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Before: [situation].
+After: [situation].
+What changed: [the one thing they can copy].
+[CTA]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>AIDA: Attention, interest, desire, action</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>[Restate the hook in new words.]
+[One surprising, specific detail.]
+[What it looks like once it's fixed.]
+[One CTA.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Quick lesson</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>[Hook restated]. The lesson: [one sentence]. [CTA]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
           <t>Three tips</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>[Number] things I wish I knew about [topic]:
 1) [tip]
@@ -3124,51 +3989,6 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Before / after</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>Before: [situation]. After: [situation]. What changed: [one thing]. [CTA]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Mistake</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>I used to [mistake]. It cost me [cost]. Now I [new habit]. Don't repeat my mistake.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Customer words</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>'[exact customer quote].' That's why we [what you do]. [CTA]</t>
-        </is>
-      </c>
-    </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="16" t="n">
         <v>6</v>
@@ -3180,7 +4000,7 @@
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>[Where you were]. [What happened]. [What you learned]. [Question for the reader]</t>
+          <t>[Where you were]. [What happened]. [What you learned]. [Question for the reader]?</t>
         </is>
       </c>
     </row>
@@ -3190,12 +4010,12 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Behind the scenes</t>
+          <t>Customer words (with permission)</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>What you didn't see: [hidden work]. This is why [result] takes [time].</t>
+          <t>"[Exact customer quote]." That's why we [what you do]. [CTA]</t>
         </is>
       </c>
     </row>
@@ -3205,12 +4025,12 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Behind the scenes</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>Honest question for [audience]: [question]? I'll reply to every comment.</t>
+          <t>What you didn't see: [the hidden work]. That's why [result] takes [time]. [CTA]</t>
         </is>
       </c>
     </row>
@@ -3220,12 +4040,12 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>Offer</t>
+          <t>Myth vs truth</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>I help [who] [get result] without [pain]. I'm taking [a real number] [clients / orders] this month. [CTA]</t>
+          <t>Myth: [common belief]. Truth: [what you've seen]. Why: [one reason]. [CTA]</t>
         </is>
       </c>
     </row>
@@ -3235,12 +4055,12 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>Myth</t>
+          <t>Honest offer</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>Myth: [common belief]. Truth: [what you've seen]. Here's why: [reason].</t>
+          <t>I help [who] [get result] without [pain]. I have room for [real number] [clients or orders] this month. [CTA]</t>
         </is>
       </c>
     </row>
@@ -3257,11 +4077,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -3286,6 +4107,11 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
+          <t>Goal</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
           <t>Call to action</t>
         </is>
       </c>
@@ -3294,9 +4120,14 @@
       <c r="A4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t>Comment '[keyword]' and I'll send you [free thing].</t>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Follow and comment [KEYWORD] and I'll DM you [free thing].</t>
         </is>
       </c>
     </row>
@@ -3304,9 +4135,14 @@
       <c r="A5" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>Save this for the next time you [situation].</t>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Reach</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Send this to a friend who [situation].</t>
         </is>
       </c>
     </row>
@@ -3314,9 +4150,14 @@
       <c r="A6" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Send this to someone who needs to [result].</t>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Saves</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Save this for the next time you [situation].</t>
         </is>
       </c>
     </row>
@@ -3324,9 +4165,14 @@
       <c r="A7" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Follow for part two.</t>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Follows</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Follow for part 2, where I [what part 2 covers]. (Only when part 2 is already filmed.)</t>
         </is>
       </c>
     </row>
@@ -3334,9 +4180,14 @@
       <c r="A8" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>DM me '[keyword]' if you want help with [problem].</t>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Sales chats</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>DM me [KEYWORD] if you want help with [problem].</t>
         </is>
       </c>
     </row>
@@ -3344,9 +4195,14 @@
       <c r="A9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>Which one are you? Tell me in the comments.</t>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Which one are you, [A] or [B]? Tell me below.</t>
         </is>
       </c>
     </row>
@@ -3354,9 +4210,14 @@
       <c r="A10" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>Link in bio to [book / order / get the free guide].</t>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Link in bio to [book, order or get the free guide]. (Use the same words on the link page.)</t>
         </is>
       </c>
     </row>
@@ -3364,9 +4225,14 @@
       <c r="A11" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>Follow if you're building [type of business] too.</t>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Proof</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Try this today and tell me how it went.</t>
         </is>
       </c>
     </row>
@@ -3374,9 +4240,14 @@
       <c r="A12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>Try this today and tell me how it goes.</t>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Trust</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Drop your [thing] below and I'll give quick feedback on the first [number]. (Then actually do it.)</t>
         </is>
       </c>
     </row>
@@ -3384,14 +4255,19 @@
       <c r="A13" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>I'm taking [a real number] [clients / orders] this week. DM me to grab a spot.</t>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>I have room for [real number] [clients or orders] this month. DM me [KEYWORD] to grab one. (Real capacity only.)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B13"/>
+  <autoFilter ref="A3:C13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -3403,7 +4279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3527,77 +4403,153 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>List</t>
         </is>
       </c>
       <c r="B9" s="24">
-        <f>COUNTIFS('My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0")</f>
+        <f>COUNTIFS('My hooks'!$C$4:$C$63,"List",'My hooks'!$F$4:$F$63,"&gt;0")</f>
         <v/>
       </c>
       <c r="C9" s="24">
-        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"List",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
         <v/>
       </c>
       <c r="D9" s="24">
-        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"List",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B10" s="24">
+        <f>COUNTIFS('My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="C10" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Result",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
           <t>Behind the scenes</t>
         </is>
       </c>
-      <c r="B10" s="24">
+      <c r="B11" s="24">
         <f>COUNTIFS('My hooks'!$C$4:$C$63,"Behind the scenes",'My hooks'!$F$4:$F$63,"&gt;0")</f>
         <v/>
       </c>
-      <c r="C10" s="24">
+      <c r="C11" s="24">
         <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Behind the scenes",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
         <v/>
       </c>
-      <c r="D10" s="24">
+      <c r="D11" s="24">
         <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Behind the scenes",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Call-out</t>
+        </is>
+      </c>
+      <c r="B12" s="24">
+        <f>COUNTIFS('My hooks'!$C$4:$C$63,"Call-out",'My hooks'!$F$4:$F$63,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="C12" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Call-out",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Call-out",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="B13" s="24">
+        <f>COUNTIFS('My hooks'!$C$4:$C$63,"Comparison",'My hooks'!$F$4:$F$63,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="C13" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Comparison",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Comparison",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>Experiment</t>
+        </is>
+      </c>
+      <c r="B14" s="24">
+        <f>COUNTIFS('My hooks'!$C$4:$C$63,"Experiment",'My hooks'!$F$4:$F$63,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="C14" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$F$4:$F$63,'My hooks'!$C$4:$C$63,"Experiment",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="24">
+        <f>IFERROR(ROUND(AVERAGEIFS('My hooks'!$H$4:$H$63,'My hooks'!$C$4:$C$63,"Experiment",'My hooks'!$F$4:$F$63,"&gt;0"),0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>YOUR WINNER</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>Hook type with the best average views</t>
         </is>
       </c>
-      <c r="B13" s="26">
-        <f>IF(COUNT($C$5:$C$10)=0,"Log some results first",INDEX($A$5:$A$10,MATCH(MAX($C$5:$C$10),$C$5:$C$10,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="B17" s="26">
+        <f>IF(COUNT($C$5:$C$14)=0,"Log some results first",INDEX($A$5:$A$14,MATCH(MAX($C$5:$C$14),$C$5:$C$14,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
         <is>
           <t>Hook type that starts the most conversations</t>
         </is>
       </c>
-      <c r="B14" s="26">
-        <f>IF(COUNT($D$5:$D$10)=0,"",INDEX($A$5:$A$10,MATCH(MAX($D$5:$D$10),$D$5:$D$10,0)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="B18" s="26">
+        <f>IF(COUNT($D$5:$D$14)=0,"",INDEX($A$5:$A$14,MATCH(MAX($D$5:$D$14),$D$5:$D$14,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Best single hook so far</t>
         </is>
       </c>
-      <c r="B15" s="27">
+      <c r="B19" s="27">
         <f>IF(COUNT('My hooks'!$F$4:$F$63)=0,"",INDEX('My hooks'!$A$4:$A$63,MATCH(MAX('My hooks'!$F$4:$F$63),'My hooks'!$F$4:$F$63,0)))</f>
         <v/>
       </c>
@@ -3889,7 +4841,7 @@
   <autoFilter ref="A3:G23"/>
   <dataValidations count="1">
     <dataValidation sqref="B4:B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Story,Mistake,Contrarian,How-to,Result,Behind the scenes"</formula1>
+      <formula1>"Story,Mistake,Contrarian,How-to,List,Result,Behind the scenes,Call-out,Comparison,Experiment"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>